<commit_message>
Fix workbook consistency defects and author approved GRC scenario decisions
</commit_message>
<xml_diff>
--- a/01-meridian-health-grc-program/artifacts/risk_register.xlsx
+++ b/01-meridian-health-grc-program/artifacts/risk_register.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Methodology" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Acceptance" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Risk Register'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Risk Register'!$A$1:$V$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Legend &amp; Methodology'!$A$1:$B$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Risk Acceptance'!$A$1:$B$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -21,8 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -82,8 +86,25 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00172B4D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00172B4D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +115,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3B61"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,7 +157,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -186,6 +212,22 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1491,7 +1533,7 @@
       </c>
       <c r="S13" s="15" t="inlineStr">
         <is>
-          <t>Add colo badge log review to quarterly physical security checklist; low residual risk given facility is being decommissioned in migration plan</t>
+          <t>Add colo badge log review to quarterly physical security checklist; Medium residual risk (score 6) given facility is being decommissioned in migration plan</t>
         </is>
       </c>
       <c r="T13" s="15" t="inlineStr">
@@ -1902,7 +1944,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="100" customHeight="1" s="11">
+    <row r="18" ht="110" customHeight="1" s="11">
       <c r="A18" s="15" t="inlineStr">
         <is>
           <t>R-014</t>
@@ -1981,7 +2023,7 @@
       </c>
       <c r="S18" s="15" t="inlineStr">
         <is>
-          <t>Monitor for abuse; Q3 rate-limiting backlog. Accepted because directory data is public and exposure does not justify remediation cost (project README). Accepter not recorded; API Platform Lead is the risk owner.</t>
+          <t>Accepted under ACC-014 by Elena Voss, COO, on 2026-03-12. Public directory data and Low residual score 2 do not justify immediate remediation cost. Monitor abuse; retain Q3 rate-limiting backlog. See Risk Acceptance for authority and conditions.</t>
         </is>
       </c>
       <c r="T18" s="15" t="inlineStr">
@@ -2199,7 +2241,7 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>20-25 — Immediate executive escalation and remediation required</t>
+          <t>15-25 — Immediate executive escalation and remediation required</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2253,7 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>10-19 — Remediation plan required within 30-60 days</t>
+          <t>10-14 — Remediation plan required within 30-60 days</t>
         </is>
       </c>
     </row>
@@ -2316,4 +2358,229 @@
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
   <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" style="11" min="1" max="1"/>
+    <col width="91" customWidth="1" style="11" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" s="11">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>MERIDIAN RISK ACCEPTANCE RECORD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1" s="11">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Scenario status</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>Fictional decision and personnel, authored for this portfolio exercise. No real executive approval is represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="11">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Acceptance ID</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>ACC-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="11">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>Related risk</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>R-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="11">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Accept with monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="11">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Accepter</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Elena Voss</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="11">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1" s="11">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Delegated authority</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Scenario risk charter delegates acceptance of Low residual operational risks involving public data to the COO. No authority to waive legal obligations or accept PHI disclosure risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1" s="11">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Decision date</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>46093</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="11">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Residual score at decision</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1" s="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Residual band</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1" s="11">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Business rationale</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>The directory is public by design. Immediate rate-limiting work would displace higher-priority PHI and access-control remediation; expected scraping exposure does not justify that cost. Q3 implementation remains in the backlog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="11">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Risk owner</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>API Platform Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1" s="11">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Conditions</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Review gateway abuse logs monthly; escalate service degradation, unexpected nonpublic data exposure, or a material change in API usage to the COO and CISO. Acceptance must be reconsidered if any condition fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1" s="11">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Scheduled review date</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>46234</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" s="11">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Acceptance expires</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1" s="11">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Review evidence</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>This record documents the March decision only. A completed July review or renewal is not supplied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1" s="11">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Closure evidence</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Rate-limiting configuration and validation of expected API behavior are required to close the remediation action. Acceptance alone does not close R-014.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>